<commit_message>
upload 1_LoadData.py but I am missing the actual link to the dataset on google set
</commit_message>
<xml_diff>
--- a/Architecture_setup_1.xlsx
+++ b/Architecture_setup_1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo PC\Documents\2026_Spring\CSC215-ArtificialIntelligence\GroupProject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4009A801-1A1F-44B7-B5A8-810014D1CAA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7898379-3EB2-4B2F-A678-0B946BB691A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31800" yWindow="2985" windowWidth="13260" windowHeight="8880" xr2:uid="{E7953A93-150F-4729-B933-EB029B147681}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" xr2:uid="{E7953A93-150F-4729-B933-EB029B147681}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="42">
   <si>
     <t># Load dataset
 # Textual: Preview dataset 1
@@ -154,6 +154,9 @@
   </si>
   <si>
     <t>architecture_setup put your name in an area you want to do in the yellow box next to the area you want to do.</t>
+  </si>
+  <si>
+    <t>John Spaugh JS</t>
   </si>
 </sst>
 </file>
@@ -353,9 +356,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -367,6 +367,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1486,252 +1489,254 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="G1" s="20" t="s">
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="G1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" s="22"/>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
-      <c r="I2" s="21"/>
-      <c r="J2" s="21"/>
+      <c r="A2" s="21"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="E2" s="22"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3" s="22"/>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="G3" s="21"/>
-      <c r="H3" s="21"/>
-      <c r="I3" s="21"/>
-      <c r="J3" s="21"/>
+      <c r="A3" s="21"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="22"/>
+      <c r="E3" s="22"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="20"/>
+      <c r="I3" s="20"/>
+      <c r="J3" s="20"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4" s="22"/>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
-      <c r="G4" s="21"/>
-      <c r="H4" s="21"/>
-      <c r="I4" s="21"/>
-      <c r="J4" s="21"/>
+      <c r="A4" s="21"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="G4" s="20"/>
+      <c r="H4" s="20"/>
+      <c r="I4" s="20"/>
+      <c r="J4" s="20"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5" s="22"/>
-      <c r="B5" s="22"/>
-      <c r="C5" s="22"/>
-      <c r="D5" s="18"/>
-      <c r="E5" s="18"/>
-      <c r="G5" s="21"/>
-      <c r="H5" s="21"/>
-      <c r="I5" s="21"/>
-      <c r="J5" s="21"/>
+      <c r="A5" s="21"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="21"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="G5" s="20"/>
+      <c r="H5" s="20"/>
+      <c r="I5" s="20"/>
+      <c r="J5" s="20"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6" s="22"/>
-      <c r="B6" s="22"/>
-      <c r="C6" s="22"/>
-      <c r="G6" s="21"/>
-      <c r="H6" s="21"/>
-      <c r="I6" s="21"/>
-      <c r="J6" s="21"/>
+      <c r="A6" s="21"/>
+      <c r="B6" s="21"/>
+      <c r="C6" s="21"/>
+      <c r="G6" s="20"/>
+      <c r="H6" s="20"/>
+      <c r="I6" s="20"/>
+      <c r="J6" s="20"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A7" s="22"/>
-      <c r="B7" s="22"/>
-      <c r="C7" s="22"/>
-      <c r="G7" s="21"/>
-      <c r="H7" s="21"/>
-      <c r="I7" s="21"/>
-      <c r="J7" s="21"/>
+      <c r="A7" s="21"/>
+      <c r="B7" s="21"/>
+      <c r="C7" s="21"/>
+      <c r="G7" s="20"/>
+      <c r="H7" s="20"/>
+      <c r="I7" s="20"/>
+      <c r="J7" s="20"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A8" s="22"/>
-      <c r="B8" s="22"/>
-      <c r="C8" s="22"/>
-      <c r="G8" s="21"/>
-      <c r="H8" s="21"/>
-      <c r="I8" s="21"/>
-      <c r="J8" s="21"/>
+      <c r="A8" s="21"/>
+      <c r="B8" s="21"/>
+      <c r="C8" s="21"/>
+      <c r="G8" s="20"/>
+      <c r="H8" s="20"/>
+      <c r="I8" s="20"/>
+      <c r="J8" s="20"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A9" s="22"/>
-      <c r="B9" s="22"/>
-      <c r="C9" s="22"/>
-      <c r="G9" s="21"/>
-      <c r="H9" s="21"/>
-      <c r="I9" s="21"/>
-      <c r="J9" s="21"/>
+      <c r="A9" s="21"/>
+      <c r="B9" s="21"/>
+      <c r="C9" s="21"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="20"/>
+      <c r="I9" s="20"/>
+      <c r="J9" s="20"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A10" s="22"/>
-      <c r="B10" s="22"/>
-      <c r="C10" s="22"/>
+      <c r="A10" s="21"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A11" s="22"/>
-      <c r="B11" s="22"/>
-      <c r="C11" s="22"/>
+      <c r="A11" s="21"/>
+      <c r="B11" s="21"/>
+      <c r="C11" s="21"/>
     </row>
     <row r="12" spans="1:11" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="22"/>
-      <c r="B12" s="22"/>
-      <c r="C12" s="22"/>
-      <c r="G12" s="20" t="s">
+      <c r="A12" s="21"/>
+      <c r="B12" s="21"/>
+      <c r="C12" s="21"/>
+      <c r="G12" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="H12" s="20"/>
-      <c r="I12" s="20"/>
-      <c r="J12" s="20"/>
-      <c r="K12" s="20"/>
+      <c r="H12" s="19"/>
+      <c r="I12" s="19"/>
+      <c r="J12" s="19"/>
+      <c r="K12" s="19"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="G13" s="20"/>
-      <c r="H13" s="20"/>
-      <c r="I13" s="20"/>
-      <c r="J13" s="20"/>
-      <c r="K13" s="20"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="G13" s="19"/>
+      <c r="H13" s="19"/>
+      <c r="I13" s="19"/>
+      <c r="J13" s="19"/>
+      <c r="K13" s="19"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="G14" s="20"/>
-      <c r="H14" s="20"/>
-      <c r="I14" s="20"/>
-      <c r="J14" s="20"/>
-      <c r="K14" s="20"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="G14" s="19"/>
+      <c r="H14" s="19"/>
+      <c r="I14" s="19"/>
+      <c r="J14" s="19"/>
+      <c r="K14" s="19"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="D15" s="18"/>
-      <c r="E15" s="18"/>
-      <c r="G15" s="20"/>
-      <c r="H15" s="20"/>
-      <c r="I15" s="20"/>
-      <c r="J15" s="20"/>
-      <c r="K15" s="20"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="G15" s="19"/>
+      <c r="H15" s="19"/>
+      <c r="I15" s="19"/>
+      <c r="J15" s="19"/>
+      <c r="K15" s="19"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="G16" s="20"/>
-      <c r="H16" s="20"/>
-      <c r="I16" s="20"/>
-      <c r="J16" s="20"/>
-      <c r="K16" s="20"/>
+      <c r="G16" s="19"/>
+      <c r="H16" s="19"/>
+      <c r="I16" s="19"/>
+      <c r="J16" s="19"/>
+      <c r="K16" s="19"/>
     </row>
     <row r="17" spans="4:11" x14ac:dyDescent="0.3">
-      <c r="G17" s="20"/>
-      <c r="H17" s="20"/>
-      <c r="I17" s="20"/>
-      <c r="J17" s="20"/>
-      <c r="K17" s="20"/>
+      <c r="G17" s="19"/>
+      <c r="H17" s="19"/>
+      <c r="I17" s="19"/>
+      <c r="J17" s="19"/>
+      <c r="K17" s="19"/>
     </row>
     <row r="18" spans="4:11" x14ac:dyDescent="0.3">
-      <c r="G18" s="20"/>
-      <c r="H18" s="20"/>
-      <c r="I18" s="20"/>
-      <c r="J18" s="20"/>
-      <c r="K18" s="20"/>
+      <c r="G18" s="19"/>
+      <c r="H18" s="19"/>
+      <c r="I18" s="19"/>
+      <c r="J18" s="19"/>
+      <c r="K18" s="19"/>
     </row>
     <row r="19" spans="4:11" x14ac:dyDescent="0.3">
-      <c r="G19" s="20"/>
-      <c r="H19" s="20"/>
-      <c r="I19" s="20"/>
-      <c r="J19" s="20"/>
-      <c r="K19" s="20"/>
+      <c r="G19" s="19"/>
+      <c r="H19" s="19"/>
+      <c r="I19" s="19"/>
+      <c r="J19" s="19"/>
+      <c r="K19" s="19"/>
     </row>
     <row r="20" spans="4:11" x14ac:dyDescent="0.3">
-      <c r="G20" s="20"/>
-      <c r="H20" s="20"/>
-      <c r="I20" s="20"/>
-      <c r="J20" s="20"/>
-      <c r="K20" s="20"/>
+      <c r="G20" s="19"/>
+      <c r="H20" s="19"/>
+      <c r="I20" s="19"/>
+      <c r="J20" s="19"/>
+      <c r="K20" s="19"/>
     </row>
     <row r="21" spans="4:11" x14ac:dyDescent="0.3">
-      <c r="G21" s="20"/>
-      <c r="H21" s="20"/>
-      <c r="I21" s="20"/>
-      <c r="J21" s="20"/>
-      <c r="K21" s="20"/>
+      <c r="G21" s="19"/>
+      <c r="H21" s="19"/>
+      <c r="I21" s="19"/>
+      <c r="J21" s="19"/>
+      <c r="K21" s="19"/>
     </row>
     <row r="22" spans="4:11" x14ac:dyDescent="0.3">
-      <c r="G22" s="20"/>
-      <c r="H22" s="20"/>
-      <c r="I22" s="20"/>
-      <c r="J22" s="20"/>
-      <c r="K22" s="20"/>
+      <c r="G22" s="19"/>
+      <c r="H22" s="19"/>
+      <c r="I22" s="19"/>
+      <c r="J22" s="19"/>
+      <c r="K22" s="19"/>
     </row>
     <row r="23" spans="4:11" x14ac:dyDescent="0.3">
-      <c r="G23" s="20"/>
-      <c r="H23" s="20"/>
-      <c r="I23" s="20"/>
-      <c r="J23" s="20"/>
-      <c r="K23" s="20"/>
+      <c r="G23" s="19"/>
+      <c r="H23" s="19"/>
+      <c r="I23" s="19"/>
+      <c r="J23" s="19"/>
+      <c r="K23" s="19"/>
     </row>
     <row r="25" spans="4:11" x14ac:dyDescent="0.3">
-      <c r="G25" s="20" t="s">
+      <c r="G25" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="H25" s="20"/>
-      <c r="I25" s="20"/>
-      <c r="J25" s="20"/>
-      <c r="K25" s="20"/>
+      <c r="H25" s="19"/>
+      <c r="I25" s="19"/>
+      <c r="J25" s="19"/>
+      <c r="K25" s="19"/>
     </row>
     <row r="26" spans="4:11" x14ac:dyDescent="0.3">
-      <c r="D26" s="18"/>
-      <c r="E26" s="18"/>
-      <c r="G26" s="20"/>
-      <c r="H26" s="20"/>
-      <c r="I26" s="20"/>
-      <c r="J26" s="20"/>
-      <c r="K26" s="20"/>
+      <c r="D26" s="22"/>
+      <c r="E26" s="22"/>
+      <c r="G26" s="19"/>
+      <c r="H26" s="19"/>
+      <c r="I26" s="19"/>
+      <c r="J26" s="19"/>
+      <c r="K26" s="19"/>
     </row>
     <row r="27" spans="4:11" x14ac:dyDescent="0.3">
-      <c r="D27" s="18"/>
-      <c r="E27" s="18"/>
-      <c r="G27" s="20"/>
-      <c r="H27" s="20"/>
-      <c r="I27" s="20"/>
-      <c r="J27" s="20"/>
-      <c r="K27" s="20"/>
+      <c r="D27" s="22"/>
+      <c r="E27" s="22"/>
+      <c r="G27" s="19"/>
+      <c r="H27" s="19"/>
+      <c r="I27" s="19"/>
+      <c r="J27" s="19"/>
+      <c r="K27" s="19"/>
     </row>
     <row r="28" spans="4:11" x14ac:dyDescent="0.3">
-      <c r="D28" s="18"/>
-      <c r="E28" s="18"/>
-      <c r="G28" s="20"/>
-      <c r="H28" s="20"/>
-      <c r="I28" s="20"/>
-      <c r="J28" s="20"/>
-      <c r="K28" s="20"/>
+      <c r="D28" s="22"/>
+      <c r="E28" s="22"/>
+      <c r="G28" s="19"/>
+      <c r="H28" s="19"/>
+      <c r="I28" s="19"/>
+      <c r="J28" s="19"/>
+      <c r="K28" s="19"/>
     </row>
     <row r="29" spans="4:11" x14ac:dyDescent="0.3">
-      <c r="G29" s="20"/>
-      <c r="H29" s="20"/>
-      <c r="I29" s="20"/>
-      <c r="J29" s="20"/>
-      <c r="K29" s="20"/>
+      <c r="G29" s="19"/>
+      <c r="H29" s="19"/>
+      <c r="I29" s="19"/>
+      <c r="J29" s="19"/>
+      <c r="K29" s="19"/>
     </row>
     <row r="30" spans="4:11" x14ac:dyDescent="0.3">
-      <c r="G30" s="20"/>
-      <c r="H30" s="20"/>
-      <c r="I30" s="20"/>
-      <c r="J30" s="20"/>
-      <c r="K30" s="20"/>
+      <c r="G30" s="19"/>
+      <c r="H30" s="19"/>
+      <c r="I30" s="19"/>
+      <c r="J30" s="19"/>
+      <c r="K30" s="19"/>
     </row>
     <row r="32" spans="4:11" x14ac:dyDescent="0.3">
       <c r="E32" s="6"/>
@@ -1743,8 +1748,8 @@
       <c r="K32" s="6"/>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A33" s="18"/>
-      <c r="B33" s="18"/>
+      <c r="A33" s="22"/>
+      <c r="B33" s="22"/>
       <c r="D33" s="4" t="s">
         <v>3</v>
       </c>
@@ -1752,15 +1757,15 @@
       <c r="M33" s="2"/>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A34" s="18"/>
-      <c r="B34" s="18"/>
+      <c r="A34" s="22"/>
+      <c r="B34" s="22"/>
       <c r="D34" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A35" s="18"/>
-      <c r="B35" s="18"/>
+      <c r="A35" s="22"/>
+      <c r="B35" s="22"/>
       <c r="D35" s="1" t="s">
         <v>5</v>
       </c>
@@ -1782,8 +1787,8 @@
       <c r="G37" s="2"/>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A39" s="18"/>
-      <c r="B39" s="18"/>
+      <c r="A39" s="22"/>
+      <c r="B39" s="22"/>
       <c r="D39" s="7" t="s">
         <v>7</v>
       </c>
@@ -1796,22 +1801,22 @@
       <c r="K39" s="2"/>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A40" s="18"/>
-      <c r="B40" s="18"/>
+      <c r="A40" s="22"/>
+      <c r="B40" s="22"/>
       <c r="D40" s="8" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A41" s="18"/>
-      <c r="B41" s="18"/>
+      <c r="A41" s="22"/>
+      <c r="B41" s="22"/>
       <c r="D41" s="8" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A42" s="18"/>
-      <c r="B42" s="18"/>
+      <c r="A42" s="22"/>
+      <c r="B42" s="22"/>
       <c r="D42" s="9" t="s">
         <v>10</v>
       </c>
@@ -1824,8 +1829,8 @@
       <c r="K42" s="6"/>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A45" s="19"/>
-      <c r="B45" s="19"/>
+      <c r="A45" s="18"/>
+      <c r="B45" s="18"/>
       <c r="D45" s="7" t="s">
         <v>11</v>
       </c>
@@ -1838,8 +1843,8 @@
       <c r="K45" s="2"/>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A46" s="19"/>
-      <c r="B46" s="19"/>
+      <c r="A46" s="18"/>
+      <c r="B46" s="18"/>
       <c r="D46" s="9" t="s">
         <v>12</v>
       </c>
@@ -1852,8 +1857,8 @@
       <c r="K46" s="6"/>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A49" s="18"/>
-      <c r="B49" s="18"/>
+      <c r="A49" s="22"/>
+      <c r="B49" s="22"/>
       <c r="D49" s="7" t="s">
         <v>13</v>
       </c>
@@ -1866,8 +1871,8 @@
       <c r="K49" s="2"/>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A50" s="18"/>
-      <c r="B50" s="18"/>
+      <c r="A50" s="22"/>
+      <c r="B50" s="22"/>
       <c r="D50" s="9" t="s">
         <v>14</v>
       </c>
@@ -1880,8 +1885,8 @@
       <c r="K50" s="6"/>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A53" s="18"/>
-      <c r="B53" s="18"/>
+      <c r="A53" s="22"/>
+      <c r="B53" s="22"/>
       <c r="D53" s="7" t="s">
         <v>15</v>
       </c>
@@ -1891,8 +1896,8 @@
       <c r="H53" s="2"/>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A54" s="18"/>
-      <c r="B54" s="18"/>
+      <c r="A54" s="22"/>
+      <c r="B54" s="22"/>
       <c r="D54" s="9" t="s">
         <v>16</v>
       </c>
@@ -1902,8 +1907,8 @@
       <c r="H54" s="6"/>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A57" s="19"/>
-      <c r="B57" s="19"/>
+      <c r="A57" s="18"/>
+      <c r="B57" s="18"/>
       <c r="D57" s="10" t="s">
         <v>17</v>
       </c>
@@ -1914,8 +1919,8 @@
       <c r="I57" s="11"/>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A60" s="18"/>
-      <c r="B60" s="18"/>
+      <c r="A60" s="22"/>
+      <c r="B60" s="22"/>
       <c r="D60" s="7" t="s">
         <v>18</v>
       </c>
@@ -1931,15 +1936,15 @@
       <c r="N60" s="2"/>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A61" s="18"/>
-      <c r="B61" s="18"/>
+      <c r="A61" s="22"/>
+      <c r="B61" s="22"/>
       <c r="D61" s="8" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A62" s="18"/>
-      <c r="B62" s="18"/>
+      <c r="A62" s="22"/>
+      <c r="B62" s="22"/>
       <c r="D62" s="8" t="s">
         <v>20</v>
       </c>
@@ -1960,8 +1965,8 @@
       <c r="N63" s="6"/>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A66" s="18"/>
-      <c r="B66" s="18"/>
+      <c r="A66" s="22"/>
+      <c r="B66" s="22"/>
       <c r="D66" s="10" t="s">
         <v>22</v>
       </c>
@@ -1972,8 +1977,8 @@
       <c r="I66" s="11"/>
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A69" s="18"/>
-      <c r="B69" s="18"/>
+      <c r="A69" s="22"/>
+      <c r="B69" s="22"/>
       <c r="D69" s="7" t="s">
         <v>23</v>
       </c>
@@ -1989,22 +1994,22 @@
       <c r="N69" s="2"/>
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A70" s="18"/>
-      <c r="B70" s="18"/>
+      <c r="A70" s="22"/>
+      <c r="B70" s="22"/>
       <c r="D70" s="8" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A71" s="18"/>
-      <c r="B71" s="18"/>
+      <c r="A71" s="22"/>
+      <c r="B71" s="22"/>
       <c r="D71" s="8" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A72" s="18"/>
-      <c r="B72" s="18"/>
+      <c r="A72" s="22"/>
+      <c r="B72" s="22"/>
       <c r="D72" s="8" t="s">
         <v>26</v>
       </c>
@@ -2030,8 +2035,8 @@
       <c r="N74" s="6"/>
     </row>
     <row r="77" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A77" s="18"/>
-      <c r="B77" s="18"/>
+      <c r="A77" s="22"/>
+      <c r="B77" s="22"/>
       <c r="D77" s="7" t="s">
         <v>29</v>
       </c>
@@ -2043,8 +2048,8 @@
       <c r="J77" s="3"/>
     </row>
     <row r="78" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A78" s="18"/>
-      <c r="B78" s="18"/>
+      <c r="A78" s="22"/>
+      <c r="B78" s="22"/>
       <c r="D78" s="9" t="s">
         <v>30</v>
       </c>
@@ -2056,8 +2061,8 @@
       <c r="J78" s="12"/>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A81" s="18"/>
-      <c r="B81" s="18"/>
+      <c r="A81" s="22"/>
+      <c r="B81" s="22"/>
       <c r="D81" s="13" t="s">
         <v>31</v>
       </c>
@@ -2068,16 +2073,16 @@
       <c r="I81" s="14"/>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A82" s="18"/>
-      <c r="B82" s="18"/>
+      <c r="A82" s="22"/>
+      <c r="B82" s="22"/>
       <c r="D82" s="8" t="s">
         <v>32</v>
       </c>
       <c r="I82" s="17"/>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A83" s="18"/>
-      <c r="B83" s="18"/>
+      <c r="A83" s="22"/>
+      <c r="B83" s="22"/>
       <c r="D83" s="8" t="s">
         <v>32</v>
       </c>
@@ -2094,8 +2099,8 @@
       <c r="I84" s="12"/>
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A87" s="18"/>
-      <c r="B87" s="18"/>
+      <c r="A87" s="22"/>
+      <c r="B87" s="22"/>
       <c r="D87" s="7" t="s">
         <v>34</v>
       </c>
@@ -2108,8 +2113,8 @@
       <c r="K87" s="2"/>
     </row>
     <row r="88" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A88" s="18"/>
-      <c r="B88" s="18"/>
+      <c r="A88" s="22"/>
+      <c r="B88" s="22"/>
       <c r="D88" s="8" t="s">
         <v>35</v>
       </c>
@@ -2127,8 +2132,8 @@
       <c r="K89" s="6"/>
     </row>
     <row r="92" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A92" s="18"/>
-      <c r="B92" s="18"/>
+      <c r="A92" s="22"/>
+      <c r="B92" s="22"/>
       <c r="D92" s="7" t="s">
         <v>37</v>
       </c>
@@ -2141,15 +2146,15 @@
       <c r="K92" s="2"/>
     </row>
     <row r="93" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A93" s="18"/>
-      <c r="B93" s="18"/>
+      <c r="A93" s="22"/>
+      <c r="B93" s="22"/>
       <c r="D93" s="8" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A94" s="18"/>
-      <c r="B94" s="18"/>
+      <c r="A94" s="22"/>
+      <c r="B94" s="22"/>
       <c r="D94" s="8" t="s">
         <v>38</v>
       </c>
@@ -2168,6 +2173,16 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="A77:B78"/>
+    <mergeCell ref="A81:B83"/>
+    <mergeCell ref="A87:B88"/>
+    <mergeCell ref="A92:B94"/>
+    <mergeCell ref="A49:B50"/>
+    <mergeCell ref="A53:B54"/>
+    <mergeCell ref="A57:B57"/>
+    <mergeCell ref="A60:B62"/>
+    <mergeCell ref="A66:B66"/>
+    <mergeCell ref="A69:B72"/>
     <mergeCell ref="A45:B46"/>
     <mergeCell ref="G25:K30"/>
     <mergeCell ref="G1:J9"/>
@@ -2178,16 +2193,6 @@
     <mergeCell ref="D26:E28"/>
     <mergeCell ref="A33:B35"/>
     <mergeCell ref="A39:B42"/>
-    <mergeCell ref="A77:B78"/>
-    <mergeCell ref="A81:B83"/>
-    <mergeCell ref="A87:B88"/>
-    <mergeCell ref="A92:B94"/>
-    <mergeCell ref="A49:B50"/>
-    <mergeCell ref="A53:B54"/>
-    <mergeCell ref="A57:B57"/>
-    <mergeCell ref="A60:B62"/>
-    <mergeCell ref="A66:B66"/>
-    <mergeCell ref="A69:B72"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>